<commit_message>
feat: implement InternalAuditController and DashboardController with CAR action reporting and verification workflows.
</commit_message>
<xml_diff>
--- a/public/tamplate-xlsx/Internal_Audit_Export_ChecksheetTamplate.xlsx
+++ b/public/tamplate-xlsx/Internal_Audit_Export_ChecksheetTamplate.xlsx
@@ -5,22 +5,22 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ICT\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\ict\www-wsl\qms\public\tamplate-xlsx\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{246820B9-BD3B-4D8D-A0A3-30012AA7C365}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6B3661D5-52DE-4F79-B2BF-2AA2443B096A}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12105" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="999999"/>
+  <calcPr calcId="191029"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="27">
   <si>
     <t>CHECKLIST AUDIT LINGKUNGAN</t>
   </si>
@@ -72,13 +72,43 @@
   </si>
   <si>
     <t>Finding</t>
+  </si>
+  <si>
+    <t>Nomor Dokumen</t>
+  </si>
+  <si>
+    <t>Departement</t>
+  </si>
+  <si>
+    <t>Manajemen</t>
+  </si>
+  <si>
+    <t>FO-08-09</t>
+  </si>
+  <si>
+    <t>Tanggal Terbit</t>
+  </si>
+  <si>
+    <t>No Revisi</t>
+  </si>
+  <si>
+    <t>Halaman</t>
+  </si>
+  <si>
+    <t>1 dari 1</t>
+  </si>
+  <si>
+    <t>01</t>
+  </si>
+  <si>
+    <t>(Tanggal di Export)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -113,6 +143,12 @@
       <color rgb="FFEF4444"/>
       <name val="Times New Roman"/>
     </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -128,7 +164,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="5">
+  <borders count="13">
     <border>
       <left/>
       <right/>
@@ -188,52 +224,132 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -243,8 +359,41 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="6" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -643,185 +792,207 @@
     <col min="7" max="7" width="18.42578125" customWidth="1"/>
     <col min="8" max="8" width="18.28515625" customWidth="1"/>
     <col min="9" max="9" width="16.7109375" customWidth="1"/>
+    <col min="11" max="11" width="18.140625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="21.140625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="2:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B2" s="6"/>
-      <c r="C2" s="6"/>
-      <c r="D2" s="6"/>
-      <c r="E2" s="2" t="s">
+      <c r="B2" s="14"/>
+      <c r="C2" s="14"/>
+      <c r="D2" s="14"/>
+      <c r="E2" s="18" t="s">
         <v>0</v>
       </c>
-      <c r="F2" s="2"/>
-      <c r="G2" s="2"/>
-      <c r="H2" s="2"/>
-      <c r="I2" s="2"/>
-      <c r="J2" s="2"/>
-      <c r="K2" s="2"/>
-      <c r="L2" s="2"/>
+      <c r="F2" s="19"/>
+      <c r="G2" s="19"/>
+      <c r="H2" s="19"/>
+      <c r="I2" s="19"/>
+      <c r="J2" s="20"/>
+      <c r="K2" s="27" t="s">
+        <v>17</v>
+      </c>
+      <c r="L2" s="27" t="s">
+        <v>20</v>
+      </c>
       <c r="M2" s="1"/>
       <c r="N2" s="1"/>
       <c r="O2" s="1"/>
     </row>
     <row r="3" spans="2:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B3" s="6"/>
-      <c r="C3" s="6"/>
-      <c r="D3" s="6"/>
-      <c r="E3" s="2"/>
-      <c r="F3" s="2"/>
-      <c r="G3" s="2"/>
-      <c r="H3" s="2"/>
-      <c r="I3" s="2"/>
-      <c r="J3" s="2"/>
-      <c r="K3" s="2"/>
-      <c r="L3" s="2"/>
+      <c r="B3" s="14"/>
+      <c r="C3" s="14"/>
+      <c r="D3" s="14"/>
+      <c r="E3" s="21"/>
+      <c r="F3" s="22"/>
+      <c r="G3" s="22"/>
+      <c r="H3" s="22"/>
+      <c r="I3" s="22"/>
+      <c r="J3" s="23"/>
+      <c r="K3" s="27" t="s">
+        <v>18</v>
+      </c>
+      <c r="L3" s="27" t="s">
+        <v>19</v>
+      </c>
       <c r="M3" s="1"/>
       <c r="N3" s="1"/>
       <c r="O3" s="1"/>
     </row>
     <row r="4" spans="2:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B4" s="6"/>
-      <c r="C4" s="6"/>
-      <c r="D4" s="6"/>
-      <c r="E4" s="2"/>
-      <c r="F4" s="2"/>
-      <c r="G4" s="2"/>
-      <c r="H4" s="2"/>
-      <c r="I4" s="2"/>
-      <c r="J4" s="2"/>
-      <c r="K4" s="2"/>
-      <c r="L4" s="2"/>
+      <c r="B4" s="14"/>
+      <c r="C4" s="14"/>
+      <c r="D4" s="14"/>
+      <c r="E4" s="21"/>
+      <c r="F4" s="22"/>
+      <c r="G4" s="22"/>
+      <c r="H4" s="22"/>
+      <c r="I4" s="22"/>
+      <c r="J4" s="23"/>
+      <c r="K4" s="27" t="s">
+        <v>21</v>
+      </c>
+      <c r="L4" s="27" t="s">
+        <v>26</v>
+      </c>
       <c r="M4" s="1"/>
       <c r="N4" s="1"/>
       <c r="O4" s="1"/>
     </row>
     <row r="5" spans="2:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B5" s="6"/>
-      <c r="C5" s="6"/>
-      <c r="D5" s="6"/>
-      <c r="E5" s="2"/>
-      <c r="F5" s="2"/>
-      <c r="G5" s="2"/>
-      <c r="H5" s="2"/>
-      <c r="I5" s="2"/>
-      <c r="J5" s="2"/>
-      <c r="K5" s="2"/>
-      <c r="L5" s="2"/>
+      <c r="B5" s="14"/>
+      <c r="C5" s="14"/>
+      <c r="D5" s="14"/>
+      <c r="E5" s="21"/>
+      <c r="F5" s="22"/>
+      <c r="G5" s="22"/>
+      <c r="H5" s="22"/>
+      <c r="I5" s="22"/>
+      <c r="J5" s="23"/>
+      <c r="K5" s="27" t="s">
+        <v>22</v>
+      </c>
+      <c r="L5" s="29" t="s">
+        <v>25</v>
+      </c>
       <c r="M5" s="1"/>
       <c r="N5" s="1"/>
       <c r="O5" s="1"/>
     </row>
     <row r="6" spans="2:15" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B6" s="6"/>
-      <c r="C6" s="6"/>
-      <c r="D6" s="6"/>
-      <c r="E6" s="2"/>
-      <c r="F6" s="2"/>
-      <c r="G6" s="2"/>
-      <c r="H6" s="2"/>
-      <c r="I6" s="2"/>
-      <c r="J6" s="2"/>
-      <c r="K6" s="2"/>
-      <c r="L6" s="2"/>
+      <c r="B6" s="14"/>
+      <c r="C6" s="14"/>
+      <c r="D6" s="14"/>
+      <c r="E6" s="24"/>
+      <c r="F6" s="25"/>
+      <c r="G6" s="25"/>
+      <c r="H6" s="25"/>
+      <c r="I6" s="25"/>
+      <c r="J6" s="26"/>
+      <c r="K6" s="27" t="s">
+        <v>23</v>
+      </c>
+      <c r="L6" s="28" t="s">
+        <v>24</v>
+      </c>
       <c r="M6" s="1"/>
       <c r="N6" s="1"/>
       <c r="O6" s="1"/>
     </row>
     <row r="7" spans="2:15" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B7" s="6"/>
-      <c r="C7" s="6"/>
-      <c r="D7" s="6"/>
-      <c r="E7" s="6"/>
-      <c r="F7" s="6"/>
-      <c r="G7" s="6"/>
-      <c r="H7" s="6"/>
-      <c r="I7" s="6"/>
-      <c r="J7" s="6"/>
-      <c r="K7" s="6"/>
-      <c r="L7" s="6"/>
-      <c r="M7" s="5"/>
-      <c r="N7" s="5"/>
-      <c r="O7" s="5"/>
+      <c r="B7" s="14"/>
+      <c r="C7" s="14"/>
+      <c r="D7" s="14"/>
+      <c r="E7" s="14"/>
+      <c r="F7" s="14"/>
+      <c r="G7" s="14"/>
+      <c r="H7" s="14"/>
+      <c r="I7" s="14"/>
+      <c r="J7" s="14"/>
+      <c r="K7" s="14"/>
+      <c r="L7" s="14"/>
+      <c r="M7" s="3"/>
+      <c r="N7" s="3"/>
+      <c r="O7" s="3"/>
     </row>
     <row r="8" spans="2:15" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B8" s="7" t="s">
+      <c r="B8" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="C8" s="7"/>
-      <c r="D8" s="7" t="s">
+      <c r="C8" s="4"/>
+      <c r="D8" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="E8" s="8"/>
-      <c r="F8" s="9"/>
-      <c r="G8" s="9"/>
-      <c r="H8" s="9"/>
-      <c r="I8" s="9"/>
-      <c r="J8" s="9"/>
-      <c r="K8" s="9"/>
-      <c r="L8" s="9"/>
-      <c r="M8" s="3"/>
-      <c r="N8" s="3"/>
-      <c r="O8" s="3"/>
+      <c r="E8" s="5"/>
+      <c r="F8" s="12"/>
+      <c r="G8" s="12"/>
+      <c r="H8" s="12"/>
+      <c r="I8" s="12"/>
+      <c r="J8" s="12"/>
+      <c r="K8" s="12"/>
+      <c r="L8" s="12"/>
+      <c r="M8" s="2"/>
+      <c r="N8" s="2"/>
+      <c r="O8" s="2"/>
     </row>
     <row r="9" spans="2:15" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B9" s="7" t="s">
+      <c r="B9" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="C9" s="7"/>
-      <c r="D9" s="7" t="s">
+      <c r="C9" s="4"/>
+      <c r="D9" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="E9" s="8"/>
-      <c r="F9" s="9"/>
-      <c r="G9" s="9"/>
-      <c r="H9" s="9"/>
-      <c r="I9" s="9"/>
-      <c r="J9" s="9"/>
-      <c r="K9" s="9"/>
-      <c r="L9" s="9"/>
-      <c r="M9" s="3"/>
-      <c r="N9" s="3"/>
-      <c r="O9" s="3"/>
+      <c r="E9" s="5"/>
+      <c r="F9" s="12"/>
+      <c r="G9" s="12"/>
+      <c r="H9" s="12"/>
+      <c r="I9" s="12"/>
+      <c r="J9" s="12"/>
+      <c r="K9" s="12"/>
+      <c r="L9" s="12"/>
+      <c r="M9" s="2"/>
+      <c r="N9" s="2"/>
+      <c r="O9" s="2"/>
     </row>
     <row r="10" spans="2:15" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B10" s="7" t="s">
+      <c r="B10" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="C10" s="7"/>
-      <c r="D10" s="7" t="s">
+      <c r="C10" s="4"/>
+      <c r="D10" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="E10" s="8"/>
-      <c r="F10" s="9"/>
-      <c r="G10" s="9"/>
-      <c r="H10" s="9"/>
-      <c r="I10" s="9"/>
-      <c r="J10" s="9"/>
-      <c r="K10" s="9"/>
-      <c r="L10" s="9"/>
-      <c r="M10" s="3"/>
-      <c r="N10" s="3"/>
-      <c r="O10" s="3"/>
+      <c r="E10" s="5"/>
+      <c r="F10" s="12"/>
+      <c r="G10" s="12"/>
+      <c r="H10" s="12"/>
+      <c r="I10" s="12"/>
+      <c r="J10" s="12"/>
+      <c r="K10" s="12"/>
+      <c r="L10" s="12"/>
+      <c r="M10" s="2"/>
+      <c r="N10" s="2"/>
+      <c r="O10" s="2"/>
     </row>
     <row r="11" spans="2:15" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B11" s="7" t="s">
+      <c r="B11" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="C11" s="7"/>
-      <c r="D11" s="7" t="s">
+      <c r="C11" s="4"/>
+      <c r="D11" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="E11" s="8"/>
-      <c r="F11" s="9"/>
-      <c r="G11" s="9"/>
-      <c r="H11" s="9"/>
-      <c r="I11" s="9"/>
-      <c r="J11" s="9"/>
-      <c r="K11" s="9"/>
-      <c r="L11" s="9"/>
-      <c r="M11" s="3"/>
-      <c r="N11" s="3"/>
-      <c r="O11" s="3"/>
+      <c r="E11" s="5"/>
+      <c r="F11" s="12"/>
+      <c r="G11" s="12"/>
+      <c r="H11" s="12"/>
+      <c r="I11" s="12"/>
+      <c r="J11" s="12"/>
+      <c r="K11" s="12"/>
+      <c r="L11" s="12"/>
+      <c r="M11" s="2"/>
+      <c r="N11" s="2"/>
+      <c r="O11" s="2"/>
     </row>
     <row r="12" spans="2:15" x14ac:dyDescent="0.25">
       <c r="B12" s="15"/>
@@ -835,98 +1006,98 @@
       <c r="J12" s="16"/>
       <c r="K12" s="16"/>
       <c r="L12" s="17"/>
-      <c r="M12" s="5"/>
-      <c r="N12" s="5"/>
-      <c r="O12" s="5"/>
+      <c r="M12" s="3"/>
+      <c r="N12" s="3"/>
+      <c r="O12" s="3"/>
     </row>
     <row r="13" spans="2:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B13" s="10" t="s">
+      <c r="B13" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="C13" s="9" t="s">
+      <c r="C13" s="12" t="s">
         <v>8</v>
       </c>
-      <c r="D13" s="9"/>
-      <c r="E13" s="9"/>
-      <c r="F13" s="9" t="s">
+      <c r="D13" s="12"/>
+      <c r="E13" s="12"/>
+      <c r="F13" s="12" t="s">
         <v>9</v>
       </c>
-      <c r="G13" s="9"/>
-      <c r="H13" s="9"/>
-      <c r="I13" s="9"/>
-      <c r="J13" s="9" t="s">
+      <c r="G13" s="12"/>
+      <c r="H13" s="12"/>
+      <c r="I13" s="12"/>
+      <c r="J13" s="12" t="s">
         <v>10</v>
       </c>
-      <c r="K13" s="9"/>
-      <c r="L13" s="9"/>
+      <c r="K13" s="12"/>
+      <c r="L13" s="12"/>
     </row>
     <row r="14" spans="2:15" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B14" s="18" t="s">
+      <c r="B14" s="13" t="s">
         <v>11</v>
       </c>
-      <c r="C14" s="18"/>
-      <c r="D14" s="18"/>
-      <c r="E14" s="18"/>
-      <c r="F14" s="18"/>
-      <c r="G14" s="18"/>
-      <c r="H14" s="18"/>
-      <c r="I14" s="18"/>
-      <c r="J14" s="18"/>
-      <c r="K14" s="18"/>
-      <c r="L14" s="18"/>
+      <c r="C14" s="13"/>
+      <c r="D14" s="13"/>
+      <c r="E14" s="13"/>
+      <c r="F14" s="13"/>
+      <c r="G14" s="13"/>
+      <c r="H14" s="13"/>
+      <c r="I14" s="13"/>
+      <c r="J14" s="13"/>
+      <c r="K14" s="13"/>
+      <c r="L14" s="13"/>
     </row>
     <row r="15" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B15" s="11">
+      <c r="B15" s="7">
         <v>1</v>
       </c>
-      <c r="C15" s="12" t="s">
+      <c r="C15" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="D15" s="12"/>
-      <c r="E15" s="12"/>
-      <c r="F15" s="13" t="s">
+      <c r="D15" s="8"/>
+      <c r="E15" s="8"/>
+      <c r="F15" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="G15" s="13"/>
-      <c r="H15" s="13"/>
-      <c r="I15" s="13"/>
-      <c r="J15" s="14" t="s">
+      <c r="G15" s="9"/>
+      <c r="H15" s="9"/>
+      <c r="I15" s="9"/>
+      <c r="J15" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="K15" s="14"/>
-      <c r="L15" s="14"/>
+      <c r="K15" s="10"/>
+      <c r="L15" s="10"/>
     </row>
     <row r="16" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B16" s="11">
+      <c r="B16" s="7">
         <v>2</v>
       </c>
-      <c r="C16" s="12" t="s">
+      <c r="C16" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="D16" s="12"/>
-      <c r="E16" s="12"/>
-      <c r="F16" s="13" t="s">
+      <c r="D16" s="8"/>
+      <c r="E16" s="8"/>
+      <c r="F16" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="G16" s="13"/>
-      <c r="H16" s="13"/>
-      <c r="I16" s="13"/>
-      <c r="J16" s="14" t="s">
+      <c r="G16" s="9"/>
+      <c r="H16" s="9"/>
+      <c r="I16" s="9"/>
+      <c r="J16" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="K16" s="14"/>
-      <c r="L16" s="14"/>
-      <c r="M16" s="4"/>
-      <c r="N16" s="4"/>
-      <c r="O16" s="4"/>
+      <c r="K16" s="10"/>
+      <c r="L16" s="10"/>
+      <c r="M16" s="11"/>
+      <c r="N16" s="11"/>
+      <c r="O16" s="11"/>
     </row>
   </sheetData>
   <mergeCells count="16">
+    <mergeCell ref="E2:J6"/>
     <mergeCell ref="C16:E16"/>
     <mergeCell ref="F16:I16"/>
     <mergeCell ref="J16:L16"/>
     <mergeCell ref="M16:O16"/>
-    <mergeCell ref="E2:L6"/>
     <mergeCell ref="F8:L11"/>
     <mergeCell ref="B14:L14"/>
     <mergeCell ref="B7:L7"/>
@@ -941,6 +1112,9 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
+  <ignoredErrors>
+    <ignoredError sqref="L5" numberStoredAsText="1"/>
+  </ignoredErrors>
   <drawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>